<commit_message>
增加一次性测全部example，gen_run.bat ，cfggen 默认print help而不是gui。
</commit_message>
<xml_diff>
--- a/example/i18n/langs/_todo_en.xlsx
+++ b/example/i18n/langs/_todo_en.xlsx
@@ -62,7 +62,8 @@
   <dimension ref="A1"/>
   <sheetFormatPr defaultRowHeight="15.0"/>
   <cols>
-    <col min="1" max="1" width="18.42578125" outlineLevel="0" customWidth="true" bestFit="true"/>
+    <col min="1" max="1" width="21.42578125" outlineLevel="0" customWidth="true" bestFit="true"/>
+    <col min="2" max="2" width="9.42578125" outlineLevel="0" customWidth="true" bestFit="true"/>
     <col min="3" max="3" width="11.42578125" outlineLevel="0" customWidth="true" bestFit="true"/>
     <col min="4" max="4" width="11.42578125" outlineLevel="0" customWidth="true" bestFit="true"/>
     <col min="5" max="5" width="11.42578125" outlineLevel="0" customWidth="true" bestFit="true"/>
@@ -206,22 +207,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>other.drop</t>
+          <t>other.ArgCaptureMode</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>Snapshot</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>comment</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>测试掉落</t>
+          <t>快照模式</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -233,22 +234,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>other.drop</t>
+          <t>other.ArgCaptureMode</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Dynamic</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>comment</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>剧情任务测试2</t>
+          <t>动态模式</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -265,7 +266,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -275,7 +276,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>通告栏掉落染色模板1</t>
+          <t>测试掉落</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -287,12 +288,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>other.loot</t>
+          <t>other.drop</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -302,7 +303,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>测试掉落</t>
+          <t>剧情任务测试2</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -314,12 +315,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>other.loot</t>
+          <t>other.drop</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -329,7 +330,7 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>小宝箱</t>
+          <t>通告栏掉落染色模板1</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -346,7 +347,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -356,7 +357,7 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>中宝箱</t>
+          <t>测试掉落</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -373,7 +374,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -383,7 +384,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>大宝箱</t>
+          <t>小宝箱</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -400,7 +401,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -410,7 +411,7 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>测试掉落2</t>
+          <t>中宝箱</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
@@ -427,7 +428,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -437,7 +438,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>剧情任务测试1</t>
+          <t>大宝箱</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -454,7 +455,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -464,7 +465,7 @@
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>剧情任务测试2</t>
+          <t>测试掉落2</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -481,7 +482,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -491,7 +492,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>通告栏掉落染色模板1</t>
+          <t>剧情任务测试1</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -508,7 +509,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -518,7 +519,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>通告栏掉落染色模板2</t>
+          <t>剧情任务测试2</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -535,7 +536,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -545,7 +546,7 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>通告栏掉落染色模板3</t>
+          <t>通告栏掉落染色模板1</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -557,22 +558,22 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>task.task</t>
+          <t>other.loot</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>9</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>name-0</t>
+          <t>name</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>和npc对话</t>
+          <t>通告栏掉落染色模板2</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -584,22 +585,22 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>task.task</t>
+          <t>other.loot</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>10</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>name-1</t>
+          <t>name</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>和npc对话</t>
+          <t>通告栏掉落染色模板3</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -616,7 +617,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -626,7 +627,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>收集物品</t>
+          <t>和npc对话</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
@@ -643,7 +644,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -653,7 +654,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>收集物品</t>
+          <t>和npc对话</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -670,7 +671,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -680,7 +681,7 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>杀怪并且收集物品</t>
+          <t>收集物品</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -697,7 +698,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -707,7 +708,7 @@
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>杀怪并且收集物品</t>
+          <t>收集物品</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -724,7 +725,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -734,7 +735,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>杀怪对话并且收集物品</t>
+          <t>杀怪并且收集物品</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
@@ -751,7 +752,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -761,7 +762,7 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>杀怪对话并且收集物品</t>
+          <t>杀怪并且收集物品</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -778,7 +779,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
@@ -788,7 +789,7 @@
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>聊天并且杀怪</t>
+          <t>杀怪对话并且收集物品</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -805,7 +806,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -815,7 +816,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>测试转义符号</t>
+          <t>杀怪对话并且收集物品</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
@@ -832,7 +833,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -842,7 +843,7 @@
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>测试</t>
+          <t>聊天并且杀怪</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -859,7 +860,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
@@ -869,7 +870,7 @@
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>测试无参数得bean</t>
+          <t>测试转义符号</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -886,7 +887,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -896,7 +897,7 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>测试2</t>
+          <t>测试</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
@@ -913,7 +914,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -923,7 +924,7 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>测试默认bean</t>
+          <t>测试无参数得bean</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -935,12 +936,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>task.task2</t>
+          <t>task.task</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -950,7 +951,7 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>测试用</t>
+          <t>测试2</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -962,22 +963,22 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>task.task2</t>
+          <t>task.task</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>name-0</t>
+          <t>name-1</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>和npc对话</t>
+          <t>测试默认bean</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
@@ -994,17 +995,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>name-1</t>
+          <t>name-0</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>和npc对话</t>
+          <t>测试用</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1021,7 +1022,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1031,7 +1032,7 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>收集物品</t>
+          <t>和npc对话</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1048,7 +1049,7 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -1058,7 +1059,7 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>收集物品</t>
+          <t>和npc对话</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1075,7 +1076,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1085,7 +1086,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>杀怪并且收集物品</t>
+          <t>收集物品</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -1102,7 +1103,7 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1112,7 +1113,7 @@
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>杀怪并且收集物品</t>
+          <t>收集物品</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
@@ -1129,7 +1130,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1139,7 +1140,7 @@
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>杀怪对话并且收集物品</t>
+          <t>杀怪并且收集物品</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1156,7 +1157,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1166,7 +1167,7 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>杀怪对话并且收集物品</t>
+          <t>杀怪并且收集物品</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1183,7 +1184,7 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -1193,7 +1194,7 @@
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>聊天并且杀怪</t>
+          <t>杀怪对话并且收集物品</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
@@ -1210,7 +1211,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1220,7 +1221,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>测试转义符号</t>
+          <t>杀怪对话并且收集物品</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -1237,7 +1238,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1247,7 +1248,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>测试</t>
+          <t>聊天并且杀怪</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -1264,7 +1265,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>7</t>
+          <t>6</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1274,7 +1275,7 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>测试无参数得bean</t>
+          <t>测试转义符号</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1291,7 +1292,7 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>7</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1301,7 +1302,7 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>测试2</t>
+          <t>测试</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1318,20 +1319,74 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>name-1</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>测试无参数得bean</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>task.task2</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
           <t>8</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>name-0</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>测试2</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t/>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>task.task2</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>8</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
         <is>
           <t>name-1</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>测试默认bean</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr">
+      <c r="E49" t="inlineStr">
         <is>
           <t/>
         </is>

</xml_diff>